<commit_message>
Add Sprint 3 FE automation suite - 138 tests passing
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/HomeData.xlsx
+++ b/src/test/resources/testdata/HomeData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local\DXC\iot-fe-automation\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Downloads\QA_Automation\s2-selenium\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACA6DEA-C3A7-453E-ACDB-15A5327C6968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460D6896-ABBB-4962-8FCD-27442AE4B485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{DCB126CA-FA20-4E2C-8C2F-44D2545692BB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{DCB126CA-FA20-4E2C-8C2F-44D2545692BB}"/>
   </bookViews>
   <sheets>
     <sheet name="home" sheetId="1" r:id="rId1"/>
@@ -161,9 +161,6 @@
     <t>Welcome Title Contains First Name</t>
   </si>
   <si>
-    <t>John</t>
-  </si>
-  <si>
     <t>TC-FE-A058</t>
   </si>
   <si>
@@ -207,6 +204,9 @@
   </si>
   <si>
     <t>Top Nav Profile Link → /profile</t>
+  </si>
+  <si>
+    <t>Mariam</t>
   </si>
 </sst>
 </file>
@@ -269,12 +269,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,14 +608,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8E6EBFC-6CA6-475D-AD3E-A8BC0C4CBA81}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -628,8 +626,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
@@ -639,8 +637,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
@@ -650,8 +648,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
@@ -661,8 +659,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
       <c r="B5" t="s">
@@ -672,8 +670,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
@@ -683,160 +681,160 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
         <v>17</v>
       </c>
       <c r="B7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
         <v>19</v>
       </c>
       <c r="B8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
         <v>21</v>
       </c>
       <c r="B9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
         <v>22</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
         <v>23</v>
       </c>
       <c r="B11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
         <v>24</v>
       </c>
       <c r="B12" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
       <c r="B13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
         <v>32</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
         <v>33</v>
       </c>
       <c r="B15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="4"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
+      <c r="B18" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="3" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
+      <c r="B19" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="4"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
+      <c r="B20" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="3" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
+      <c r="B21" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="C21" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="3" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
+      <c r="B22" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
+      <c r="B23" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>43</v>
+      <c r="C23" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>